<commit_message>
excel tempos de vida
</commit_message>
<xml_diff>
--- a/Cenarios_LC_completo.xlsx
+++ b/Cenarios_LC_completo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lifecycle\LC-eureka\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\codigo\LC-eureka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_E07A1F3BD26EB21EEB109CD75D322E3B3D045751" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534A7768-5663-4A98-926A-2F987D752F70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="316">
   <si>
     <t>Fruto</t>
   </si>
@@ -1009,6 +1009,7 @@
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1493,6 +1494,9 @@
       <c r="M6" s="3" t="s">
         <v>21</v>
       </c>
+      <c r="N6" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="7" spans="3:14" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C7" s="4" t="s">
@@ -1525,6 +1529,9 @@
       <c r="M7" s="5" t="s">
         <v>27</v>
       </c>
+      <c r="N7" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="8" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C8" s="4" t="s">
@@ -1557,6 +1564,9 @@
       <c r="M8" s="3" t="s">
         <v>37</v>
       </c>
+      <c r="N8" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="9" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C9" s="4" t="s">
@@ -1589,6 +1599,9 @@
       <c r="M9" s="3" t="s">
         <v>43</v>
       </c>
+      <c r="N9" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="10" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C10" s="4" t="s">
@@ -1621,6 +1634,9 @@
       <c r="M10" s="3" t="s">
         <v>52</v>
       </c>
+      <c r="N10" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="11" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C11" s="4" t="s">
@@ -1653,6 +1669,9 @@
       <c r="M11" s="5" t="s">
         <v>58</v>
       </c>
+      <c r="N11" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="12" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C12" s="4" t="s">
@@ -1685,6 +1704,9 @@
       <c r="M12" s="3" t="s">
         <v>66</v>
       </c>
+      <c r="N12" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="13" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C13" s="4" t="s">
@@ -1717,6 +1739,9 @@
       <c r="M13" s="3" t="s">
         <v>70</v>
       </c>
+      <c r="N13" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="14" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C14" s="4" t="s">
@@ -1749,6 +1774,9 @@
       <c r="M14" s="3" t="s">
         <v>79</v>
       </c>
+      <c r="N14" s="7" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="15" spans="3:14" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C15" s="4" t="s">
@@ -1781,8 +1809,11 @@
       <c r="M15" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="16" spans="3:14" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="N15" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="16" spans="3:14" ht="44" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C16" s="4" t="s">
         <v>83</v>
       </c>
@@ -1813,8 +1844,11 @@
       <c r="M16" s="3" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="17" spans="3:14" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="N16" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="3:14" ht="42.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C17" s="6" t="s">
         <v>93</v>
       </c>

</xml_diff>